<commit_message>
Add Xavier Racine Bechard lead to missed-leads tracker
Second entry: REALTOR.ca inquiry (Jun 11, 2026) for 12 Crocus Hill Lane.
FUB task was created but no correspondence sent since the original message.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjASex5CkM7x1T5s7pqGA6
</commit_message>
<xml_diff>
--- a/Missed_Leads_Tracker.xlsx
+++ b/Missed_Leads_Tracker.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -614,6 +614,63 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Xavier Racine Bechard</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>xavier.racine.bechard@gmail.com</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>12 Crocus Hill Lane, Whitehorse North, Yukon Y1A7A2 (MLS #17130)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Requested more information about the property, asked whether a visit/showing is possible, and said he is curious about the loan (financing). Inquiry came in via REALTOR.ca.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>General inquiry submitted through REALTOR.ca asking for more info, a possible visit, and about the loan. A task was created in Follow Up Boss (FUB), but no correspondence has been sent since.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Missed - FUB Task Created, No Response Sent</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Reply with property details and MLS info, offer a showing, and answer the financing/loan question. Close out the open FUB task once contacted.</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>FUB task created but never followed up. Note: a prior purchase contract on this property was rescinded (May 2026), so it may be available.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Clean tracker notes and widen columns
Remove scam/identity-verification commentary so entries carry only the
provided lead info, and widen columns for readability.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjASex5CkM7x1T5s7pqGA6
</commit_message>
<xml_diff>
--- a/Missed_Leads_Tracker.xlsx
+++ b/Missed_Leads_Tracker.xlsx
@@ -48,7 +48,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -58,11 +58,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -100,9 +95,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -473,17 +465,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,7 +492,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Lead Name</t>
@@ -553,11 +545,11 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Flags / Notes</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="90" customHeight="1">
+    <row r="5" ht="105" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Tik Mad</t>
@@ -575,7 +567,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Relocating with partner; expressed strong interest in the property. Requested a Zoom video meeting (specifically on a Windows device) to discuss questions, saying phone calls have connection issues.</t>
+          <t>Relocating with partner; interested in the property. Requested a Zoom video meeting on a Windows device to discuss questions, noting phone calls can have connection issues.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -605,16 +597,12 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Decide: send screening/qualifying questions before scheduling, OR share Zoom availability. Verify identity first.</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Possible rental-scam pattern: unvetted 'relocating' prospect pushing to move to Zoom on a 'Windows device' citing phone-call issues. Screen before investing time.</t>
-        </is>
-      </c>
+          <t>Share Zoom availability and schedule the video meeting.</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
     </row>
-    <row r="6" ht="90" customHeight="1">
+    <row r="6" ht="105" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Xavier Racine Bechard</t>
@@ -665,9 +653,9 @@
           <t>Reply with property details and MLS info, offer a showing, and answer the financing/loan question. Close out the open FUB task once contacted.</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>FUB task created but never followed up. Note: a prior purchase contract on this property was rescinded (May 2026), so it may be available.</t>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>FUB task created but no correspondence since the original email.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Casey, Taylor, Steve, and Fr. John to missed-leads tracker
Log four more missed leads with facts only: Casey Wrightmeyer (2102
Centennial open-house question), Taylor Champeval (Marsh Lake evaluation
+ Mendenhall interest), Steve Osborne (trailer/small-home inquiry), and
Fr. John / St. Nikolai Orthodox Mission (religious-assembly-zoned buy/rent).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjASex5CkM7x1T5s7pqGA6
</commit_message>
<xml_diff>
--- a/Missed_Leads_Tracker.xlsx
+++ b/Missed_Leads_Tracker.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -659,6 +659,226 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="105" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Casey Wrightmeyer</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>cwrightmeyer@csnwhitehorse.com</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>2102 Centennial Street, Whitehorse, Yukon Y1A3Z7 (MLS #17347)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Submitted a showing request via REALTOR.ca, then followed up asking how long the open house runs, noting he doesn't get off work until 5pm.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Casey asked how long the open house lasts (doesn't get off work until 5pm). No reply was sent.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Missed - No Response Sent</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Reply about the open house / showing timing.</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="105" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Champeval</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>taylorchampeval@gmail.com  |  867-322-1976</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Marsh Lake home (evaluation) + interested in a Mendenhall property under conditional offer</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Taylor and her husband want their Marsh Lake home appraised/evaluated. Interested in a Mendenhall property currently under a conditional offer; want to be ready in case it falls through.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Taylor's last message clarified which house is theirs ("that was the one down below our house"). No reply was sent after.</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Missed - No Response Sent; Not in FUB</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Confirm the correct property and book the Marsh Lake home evaluation.</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Not in FUB. Phone: 867-322-1976.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="105" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Steve Osborne</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>stevedeb.osborne@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>95-986 Range Road (MLS #17171) - trailer; open to any 2-3 bdrm trailer in Northlands or Takhini trailer park; possibly a small home ~$500K</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Interested in the trailer listing or any 2- or 3-bedroom trailer in Northlands or Takhini trailer park. Could also be interested in a small home around $500K.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Inbound inquiry via REALTOR.ca / Kijiji. No reply was ever sent.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Missed - No Response Sent; Not in FUB</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Reply with matching trailer / small-home options.</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Not in FUB. Inquiry came via REALTOR.ca / Kijiji.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="105" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Fr. John (St. Nikolai Orthodox Mission)</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>grybas@northwestel.net</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Seeking 1200-1600 sq ft single-level on a lot zoned for religious assemblies (re: 2001 Centennial St)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Church/mission looking for a 1200-1600 sq ft single-level home where interior walls can be removed, on a lot zoned for religious assemblies. Open to buy or rent anywhere in the City zoned for religious assembly. Also seeking a ~1200-1600 sq ft rental zoned for a church while waiting to purchase. Noted 2001 Centennial too big; 1602 was close but topography and a non-legal suite didn't work.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Followed up saying they are open to buy or rent anywhere in the City zoned for religious assembly, and asked to be kept in mind. No reply was sent.</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Missed - No Response Sent</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Reply and keep an eye out for religious-assembly-zoned buy/rent options.</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Rob Drapeau to missed-leads tracker
Seventh entry: met in person May 11, sent supporting docs for 106
Normandy, 1602 Centennial, and 56 Topaz; no correspondence since.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjASex5CkM7x1T5s7pqGA6
</commit_message>
<xml_diff>
--- a/Missed_Leads_Tracker.xlsx
+++ b/Missed_Leads_Tracker.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -879,6 +879,59 @@
       </c>
       <c r="K10" s="4" t="inlineStr"/>
     </row>
+    <row r="11" ht="105" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Rob Drapeau</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>robert.drapeau@rcmp-grc.gc.ca</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>106 Normandy, 1602 Centennial &amp; 56 Topaz</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Britt met with Rob and sent supporting documents for 106 Normandy, 1602 Centennial, and 56 Topaz.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Britt wrote to Rob on May 11 ("It was great meeting you today!") attaching supporting documents for all three properties. No correspondence since.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Missed - No Response Since May 11</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Follow up with Rob on the three properties.</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Matthew Van Loon to missed-leads tracker
Eighth entry: May 11 inquiry for 908 Hotsprings Road, in FUB assigned to
Brittany Widrig, no response sent.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjASex5CkM7x1T5s7pqGA6
</commit_message>
<xml_diff>
--- a/Missed_Leads_Tracker.xlsx
+++ b/Missed_Leads_Tracker.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -932,6 +932,63 @@
       </c>
       <c r="K11" s="4" t="inlineStr"/>
     </row>
+    <row r="12" ht="105" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Matthew Van Loon</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Vanloonmatt@hotmail.com</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>908 Hotsprings Road, Whitehorse North, Yukon Y1A7A2</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Requested more information about 908 Hotsprings Road. Added to FUB, assigned to Brittany Widrig.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Wrote on May 11 asking for more information about 908 Hotsprings Road. No response.</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Missed - No Response Sent</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Reply with more information on 908 Hotsprings Road.</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>In FUB, assigned to Brittany Widrig.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Enrich Rob Drapeau entry with second email and showing details
Same lead (not a duplicate): add Radrapeau@gmail.com alongside the RCMP
address, and note the in-person 106 Normandy showing plus the requested
Topaz showing.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjASex5CkM7x1T5s7pqGA6
</commit_message>
<xml_diff>
--- a/Missed_Leads_Tracker.xlsx
+++ b/Missed_Leads_Tracker.xlsx
@@ -887,7 +887,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>robert.drapeau@rcmp-grc.gc.ca</t>
+          <t>Radrapeau@gmail.com  |  robert.drapeau@rcmp-grc.gc.ca</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Britt met with Rob and sent supporting documents for 106 Normandy, 1602 Centennial, and 56 Topaz.</t>
+          <t>Realtor.ca lead who inquired about all three properties. Britt showed him 106 Normandy Drive in person, sent supporting documents for 106 Normandy, 1602 Centennial, and 56 Topaz, and requested a Topaz showing for the next day at 4 PM.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Britt wrote to Rob on May 11 ("It was great meeting you today!") attaching supporting documents for all three properties. No correspondence since.</t>
+          <t>Britt wrote to Rob on May 11 ("It was great meeting you today!") attaching supporting documents for all three properties, after showing him 106 Normandy and lining up a Topaz showing for the next day at 4 PM. No correspondence since.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">

</xml_diff>